<commit_message>
feat: optimize Excel import performance and fix visibility bugs
</commit_message>
<xml_diff>
--- a/Inventaire_Parc.xlsx
+++ b/Inventaire_Parc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rdenimal\Documents\App_Novadis\scan_CLT_SRV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CDCC05-23F2-4314-8A4E-0C818F3E0CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDF98C8-53C1-4F8D-BD06-1D55B9F6B25F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16605" windowWidth="29040" windowHeight="15720" tabRatio="867" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2062,7 +2062,7 @@
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2249,13 +2249,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2870,7 +2863,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="193">
+  <cellXfs count="189">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
@@ -3206,12 +3199,120 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3222,118 +3323,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3400,13 +3390,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3414,15 +3397,7 @@
     <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="42">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="37">
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -3820,38 +3795,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -5810,11 +5753,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tableau23" displayName="Tableau23" ref="A1:E5" totalsRowShown="0" headerRowDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tableau23" displayName="Tableau23" ref="A1:E5" totalsRowShown="0" headerRowDxfId="32">
   <autoFilter ref="A1:E5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="DATE" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{5DEF4043-5815-4D96-A476-B2BE874CB19C}" name="INTERVENANTS" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="DATE" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{5DEF4043-5815-4D96-A476-B2BE874CB19C}" name="INTERVENANTS" dataDxfId="30"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="COMMENTAIRES"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Installateur"/>
     <tableColumn id="4" xr3:uid="{71E13FC5-5F51-4DD4-A539-65598EAA9C9F}" name="Num CC "/>
@@ -5824,53 +5767,48 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A95A6209-1B70-443E-94DD-EC0280EE8FAA}" name="Tableau1614" displayName="Tableau1614" ref="A1:F8" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A95A6209-1B70-443E-94DD-EC0280EE8FAA}" name="Tableau1614" displayName="Tableau1614" ref="A1:F8" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="A1:F8" xr:uid="{A95A6209-1B70-443E-94DD-EC0280EE8FAA}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{10302989-DA47-4F9A-831D-E2974FA029B3}" name="ANNEE" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{ADF607E8-2332-4ED7-B4B1-1E4AE95D9922}" name="MAINTENANCE" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{346F14B9-6F07-4EED-9ACF-DC92F9BDBB9F}" name="APPLICATIF (SUPP)" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{D168D9DB-08C6-41FD-A4CE-A8BBF2B957ED}" name="ACCES AU SUPPORT" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{CF36272B-8461-4E86-BFC8-4B628913DA06}" name="INTERVENTION CORRECTIVE" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{0487574F-CC11-4397-AFB0-175DD4DD25E4}" name="COMMENTAIRES" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{10302989-DA47-4F9A-831D-E2974FA029B3}" name="ANNEE" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{ADF607E8-2332-4ED7-B4B1-1E4AE95D9922}" name="MAINTENANCE" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{346F14B9-6F07-4EED-9ACF-DC92F9BDBB9F}" name="APPLICATIF (SUPP)" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{D168D9DB-08C6-41FD-A4CE-A8BBF2B957ED}" name="ACCES AU SUPPORT" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{CF36272B-8461-4E86-BFC8-4B628913DA06}" name="INTERVENTION CORRECTIVE" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{0487574F-CC11-4397-AFB0-175DD4DD25E4}" name="COMMENTAIRES" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tableau10" displayName="Tableau10" ref="A1:G66" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
-  <autoFilter ref="A1:G66" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="NOM" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Colonne1" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{3B4276FE-F454-4385-B5FB-7FB1AAFE58E5}" name="SRV-CA-STDO" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{7D4F944F-968E-4F71-B92B-707F879FF2B6}" name="CLT-CA-STDO" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{29E965B0-9881-4424-8BF7-507FDD71D137}" name="SRV-VID-STDO" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{B03954D5-5D65-41DD-B99E-DE2FE05FD7BF}" name="CLT-VID-STDO" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{1F7D1893-8690-4501-B5A3-FE1CB0855975}" name="LAPTOP-77OIEFCV" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tableau10" displayName="Tableau10" ref="A1:B66" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+  <autoFilter ref="A1:B66" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="NOM" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Colonne1" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tableau1" displayName="Tableau1" ref="A1:F33" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tableau1" displayName="Tableau1" ref="A1:F33" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20">
   <autoFilter ref="A1:F33" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="Système" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="Identifiant" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="Mot de passe" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="Logiciels / Equipements" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{247F378F-624F-4E7F-91A0-E54FF940766A}" name="Profil" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{6A6A4012-25DA-49C8-9179-3464CF503144}" name="Commentaires" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="Système" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="Identifiant" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="Mot de passe" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="Logiciels / Equipements" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{247F378F-624F-4E7F-91A0-E54FF940766A}" name="Profil" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{6A6A4012-25DA-49C8-9179-3464CF503144}" name="Commentaires" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Tableau9" displayName="Tableau9" ref="A1:K24" totalsRowShown="0" headerRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Tableau9" displayName="Tableau9" ref="A1:K24" totalsRowShown="0" headerRowDxfId="12">
   <autoFilter ref="A1:K24" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="NOM DE LA CAMERA"/>
@@ -5880,7 +5818,7 @@
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0700-000011000000}" name="NUMERO DE SERIE"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="FIRMWARE"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="ADRESSE IP"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="MASQUE DE SOUS-RESEAU" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="MASQUE DE SOUS-RESEAU" dataDxfId="11"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="PASSERELLE"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="Serveur d'enregistrement"/>
     <tableColumn id="9" xr3:uid="{9D2A4D7A-4F3C-4221-8885-CC96E6ED66BD}" name="DM associé"/>
@@ -5890,14 +5828,14 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tableau7" displayName="Tableau7" ref="A1:F7" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tableau7" displayName="Tableau7" ref="A1:F7" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Equipement" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{E4E49256-DD14-4B29-8430-F91236906A84}" name="Libellé" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="ADRESSE IP" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Numéro de port" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Version Centrale" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{1E3BE692-70B3-4C08-921B-594FFF56DE07}" name="Commentaires" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Equipement" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{E4E49256-DD14-4B29-8430-F91236906A84}" name="Libellé" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="ADRESSE IP" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Numéro de port" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Version Centrale" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{1E3BE692-70B3-4C08-921B-594FFF56DE07}" name="Commentaires" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6222,14 +6160,14 @@
       <c r="A1" s="90" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="125"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
+      <c r="F1" s="125"/>
+      <c r="G1" s="125"/>
+      <c r="H1" s="125"/>
+      <c r="I1" s="125"/>
       <c r="J1" s="91" t="s">
         <v>1</v>
       </c>
@@ -6238,62 +6176,62 @@
       <c r="A2" s="92" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="161"/>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="161"/>
-      <c r="I2" s="161"/>
+      <c r="B2" s="126"/>
+      <c r="C2" s="126"/>
+      <c r="D2" s="126"/>
+      <c r="E2" s="126"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="126"/>
+      <c r="H2" s="126"/>
+      <c r="I2" s="126"/>
     </row>
     <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="162"/>
-      <c r="C3" s="162"/>
-      <c r="D3" s="162"/>
-      <c r="E3" s="162"/>
-      <c r="F3" s="162"/>
-      <c r="G3" s="162"/>
-      <c r="H3" s="162"/>
-      <c r="I3" s="162"/>
+      <c r="B3" s="127"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="127"/>
+      <c r="E3" s="127"/>
+      <c r="F3" s="127"/>
+      <c r="G3" s="127"/>
+      <c r="H3" s="127"/>
+      <c r="I3" s="127"/>
     </row>
     <row r="4" spans="1:11" ht="109.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="163"/>
-      <c r="C4" s="163"/>
-      <c r="D4" s="163"/>
-      <c r="E4" s="163"/>
-      <c r="F4" s="163"/>
-      <c r="G4" s="163"/>
-      <c r="H4" s="163"/>
-      <c r="I4" s="163"/>
+      <c r="B4" s="128"/>
+      <c r="C4" s="128"/>
+      <c r="D4" s="128"/>
+      <c r="E4" s="128"/>
+      <c r="F4" s="128"/>
+      <c r="G4" s="128"/>
+      <c r="H4" s="128"/>
+      <c r="I4" s="128"/>
     </row>
     <row r="5" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="164" t="s">
+      <c r="A5" s="129" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="167" t="s">
+      <c r="B5" s="132" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="167"/>
-      <c r="D5" s="167" t="s">
+      <c r="C5" s="132"/>
+      <c r="D5" s="132" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="167"/>
-      <c r="F5" s="167" t="s">
+      <c r="E5" s="132"/>
+      <c r="F5" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="167"/>
-      <c r="H5" s="167"/>
-      <c r="I5" s="167"/>
+      <c r="G5" s="132"/>
+      <c r="H5" s="132"/>
+      <c r="I5" s="132"/>
     </row>
     <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="165"/>
+      <c r="A6" s="130"/>
       <c r="B6" s="95" t="s">
         <v>9</v>
       </c>
@@ -6312,7 +6250,7 @@
       <c r="I6" s="94"/>
     </row>
     <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="165"/>
+      <c r="A7" s="130"/>
       <c r="B7" s="95" t="s">
         <v>13</v>
       </c>
@@ -6331,7 +6269,7 @@
       <c r="I7" s="94"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="165"/>
+      <c r="A8" s="130"/>
       <c r="B8" s="95" t="s">
         <v>16</v>
       </c>
@@ -6350,7 +6288,7 @@
       <c r="I8" s="94"/>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="166"/>
+      <c r="A9" s="131"/>
       <c r="B9" s="95" t="s">
         <v>18</v>
       </c>
@@ -6372,16 +6310,16 @@
       <c r="A10" s="92" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="154" t="s">
+      <c r="B10" s="139" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="155"/>
-      <c r="D10" s="155"/>
-      <c r="E10" s="155"/>
-      <c r="F10" s="155"/>
-      <c r="G10" s="155"/>
-      <c r="H10" s="155"/>
-      <c r="I10" s="155"/>
+      <c r="C10" s="140"/>
+      <c r="D10" s="140"/>
+      <c r="E10" s="140"/>
+      <c r="F10" s="140"/>
+      <c r="G10" s="140"/>
+      <c r="H10" s="140"/>
+      <c r="I10" s="140"/>
       <c r="J10" s="96"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -6437,14 +6375,14 @@
       <c r="A14" s="90" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="156"/>
-      <c r="C14" s="156"/>
-      <c r="D14" s="156"/>
-      <c r="E14" s="156"/>
-      <c r="F14" s="156"/>
-      <c r="G14" s="156"/>
-      <c r="H14" s="156"/>
-      <c r="I14" s="156"/>
+      <c r="B14" s="141"/>
+      <c r="C14" s="141"/>
+      <c r="D14" s="141"/>
+      <c r="E14" s="141"/>
+      <c r="F14" s="141"/>
+      <c r="G14" s="141"/>
+      <c r="H14" s="141"/>
+      <c r="I14" s="141"/>
       <c r="J14" s="103"/>
       <c r="K14" s="104"/>
     </row>
@@ -6454,126 +6392,126 @@
       <c r="K15" s="104"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="148" t="s">
+      <c r="A16" s="154" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="147" t="s">
+      <c r="B16" s="142" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="147"/>
-      <c r="D16" s="147" t="s">
+      <c r="C16" s="142"/>
+      <c r="D16" s="142" t="s">
         <v>30</v>
       </c>
-      <c r="E16" s="147"/>
+      <c r="E16" s="142"/>
       <c r="F16" s="100" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="157" t="s">
+      <c r="G16" s="143" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="158"/>
-      <c r="I16" s="159"/>
+      <c r="H16" s="144"/>
+      <c r="I16" s="145"/>
       <c r="J16" s="103"/>
       <c r="K16" s="104"/>
     </row>
     <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="149"/>
-      <c r="B17" s="152"/>
-      <c r="C17" s="153"/>
-      <c r="D17" s="151"/>
-      <c r="E17" s="151"/>
+      <c r="A17" s="155"/>
+      <c r="B17" s="137"/>
+      <c r="C17" s="138"/>
+      <c r="D17" s="133"/>
+      <c r="E17" s="133"/>
       <c r="F17" s="114"/>
-      <c r="G17" s="144"/>
-      <c r="H17" s="145"/>
-      <c r="I17" s="146"/>
+      <c r="G17" s="134"/>
+      <c r="H17" s="135"/>
+      <c r="I17" s="136"/>
     </row>
     <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="149"/>
-      <c r="B18" s="152"/>
-      <c r="C18" s="153"/>
-      <c r="D18" s="151"/>
-      <c r="E18" s="151"/>
+      <c r="A18" s="155"/>
+      <c r="B18" s="137"/>
+      <c r="C18" s="138"/>
+      <c r="D18" s="133"/>
+      <c r="E18" s="133"/>
       <c r="F18" s="114"/>
-      <c r="G18" s="144"/>
-      <c r="H18" s="145"/>
-      <c r="I18" s="146"/>
+      <c r="G18" s="134"/>
+      <c r="H18" s="135"/>
+      <c r="I18" s="136"/>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="149"/>
-      <c r="B19" s="152"/>
-      <c r="C19" s="153"/>
-      <c r="D19" s="151"/>
-      <c r="E19" s="151"/>
+      <c r="A19" s="155"/>
+      <c r="B19" s="137"/>
+      <c r="C19" s="138"/>
+      <c r="D19" s="133"/>
+      <c r="E19" s="133"/>
       <c r="F19" s="114"/>
-      <c r="G19" s="144"/>
-      <c r="H19" s="145"/>
-      <c r="I19" s="146"/>
+      <c r="G19" s="134"/>
+      <c r="H19" s="135"/>
+      <c r="I19" s="136"/>
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="149"/>
-      <c r="B20" s="152"/>
-      <c r="C20" s="153"/>
-      <c r="D20" s="151"/>
-      <c r="E20" s="151"/>
+      <c r="A20" s="155"/>
+      <c r="B20" s="137"/>
+      <c r="C20" s="138"/>
+      <c r="D20" s="133"/>
+      <c r="E20" s="133"/>
       <c r="F20" s="114"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="145"/>
-      <c r="I20" s="146"/>
+      <c r="G20" s="134"/>
+      <c r="H20" s="135"/>
+      <c r="I20" s="136"/>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="149"/>
-      <c r="B21" s="152"/>
-      <c r="C21" s="153"/>
-      <c r="D21" s="151"/>
-      <c r="E21" s="151"/>
+      <c r="A21" s="155"/>
+      <c r="B21" s="137"/>
+      <c r="C21" s="138"/>
+      <c r="D21" s="133"/>
+      <c r="E21" s="133"/>
       <c r="F21" s="114"/>
-      <c r="G21" s="144"/>
-      <c r="H21" s="145"/>
-      <c r="I21" s="146"/>
+      <c r="G21" s="134"/>
+      <c r="H21" s="135"/>
+      <c r="I21" s="136"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="149"/>
-      <c r="B22" s="151"/>
-      <c r="C22" s="151"/>
-      <c r="D22" s="143"/>
-      <c r="E22" s="143"/>
+      <c r="A22" s="155"/>
+      <c r="B22" s="133"/>
+      <c r="C22" s="133"/>
+      <c r="D22" s="146"/>
+      <c r="E22" s="146"/>
       <c r="F22" s="114"/>
-      <c r="G22" s="144"/>
-      <c r="H22" s="145"/>
-      <c r="I22" s="146"/>
+      <c r="G22" s="134"/>
+      <c r="H22" s="135"/>
+      <c r="I22" s="136"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="149"/>
-      <c r="B23" s="151"/>
-      <c r="C23" s="151"/>
-      <c r="D23" s="143"/>
-      <c r="E23" s="143"/>
+      <c r="A23" s="155"/>
+      <c r="B23" s="133"/>
+      <c r="C23" s="133"/>
+      <c r="D23" s="146"/>
+      <c r="E23" s="146"/>
       <c r="F23" s="114"/>
-      <c r="G23" s="144"/>
-      <c r="H23" s="145"/>
-      <c r="I23" s="146"/>
+      <c r="G23" s="134"/>
+      <c r="H23" s="135"/>
+      <c r="I23" s="136"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="149"/>
-      <c r="B24" s="142"/>
-      <c r="C24" s="142"/>
-      <c r="D24" s="143"/>
-      <c r="E24" s="143"/>
+      <c r="A24" s="155"/>
+      <c r="B24" s="147"/>
+      <c r="C24" s="147"/>
+      <c r="D24" s="146"/>
+      <c r="E24" s="146"/>
       <c r="F24" s="114"/>
-      <c r="G24" s="144"/>
-      <c r="H24" s="145"/>
-      <c r="I24" s="146"/>
+      <c r="G24" s="134"/>
+      <c r="H24" s="135"/>
+      <c r="I24" s="136"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="150"/>
-      <c r="B25" s="142"/>
-      <c r="C25" s="142"/>
-      <c r="D25" s="143"/>
-      <c r="E25" s="143"/>
+      <c r="A25" s="156"/>
+      <c r="B25" s="147"/>
+      <c r="C25" s="147"/>
+      <c r="D25" s="146"/>
+      <c r="E25" s="146"/>
       <c r="F25" s="114"/>
-      <c r="G25" s="144"/>
-      <c r="H25" s="145"/>
-      <c r="I25" s="146"/>
+      <c r="G25" s="134"/>
+      <c r="H25" s="135"/>
+      <c r="I25" s="136"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="22"/>
@@ -6586,13 +6524,13 @@
       <c r="H26" s="23"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="130" t="s">
+      <c r="A27" s="148" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="139" t="s">
+      <c r="B27" s="149" t="s">
         <v>34</v>
       </c>
-      <c r="C27" s="140"/>
+      <c r="C27" s="150"/>
       <c r="D27" s="100" t="s">
         <v>35</v>
       </c>
@@ -6602,297 +6540,297 @@
       <c r="F27" s="113" t="s">
         <v>37</v>
       </c>
-      <c r="G27" s="147" t="s">
+      <c r="G27" s="142" t="s">
         <v>38</v>
       </c>
-      <c r="H27" s="147"/>
-      <c r="I27" s="147"/>
+      <c r="H27" s="142"/>
+      <c r="I27" s="142"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="130"/>
-      <c r="B28" s="134" t="s">
+      <c r="A28" s="148"/>
+      <c r="B28" s="151" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="135"/>
+      <c r="C28" s="152"/>
       <c r="D28" s="116"/>
       <c r="E28" s="93"/>
       <c r="F28" s="93"/>
-      <c r="G28" s="126"/>
-      <c r="H28" s="126"/>
-      <c r="I28" s="126"/>
+      <c r="G28" s="153"/>
+      <c r="H28" s="153"/>
+      <c r="I28" s="153"/>
     </row>
     <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="130"/>
-      <c r="B29" s="134" t="s">
+      <c r="A29" s="148"/>
+      <c r="B29" s="151" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="135"/>
+      <c r="C29" s="152"/>
       <c r="D29" s="116"/>
       <c r="E29" s="93"/>
       <c r="F29" s="93"/>
-      <c r="G29" s="126"/>
-      <c r="H29" s="126"/>
-      <c r="I29" s="126"/>
+      <c r="G29" s="153"/>
+      <c r="H29" s="153"/>
+      <c r="I29" s="153"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="130"/>
-      <c r="B30" s="134" t="s">
+      <c r="A30" s="148"/>
+      <c r="B30" s="151" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="135"/>
+      <c r="C30" s="152"/>
       <c r="D30" s="116"/>
       <c r="E30" s="93"/>
       <c r="F30" s="93"/>
-      <c r="G30" s="126"/>
-      <c r="H30" s="126"/>
-      <c r="I30" s="126"/>
+      <c r="G30" s="153"/>
+      <c r="H30" s="153"/>
+      <c r="I30" s="153"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="130"/>
-      <c r="B31" s="134" t="s">
+      <c r="A31" s="148"/>
+      <c r="B31" s="151" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="135"/>
+      <c r="C31" s="152"/>
       <c r="D31" s="116"/>
       <c r="E31" s="93"/>
       <c r="F31" s="93"/>
-      <c r="G31" s="126"/>
-      <c r="H31" s="126"/>
-      <c r="I31" s="126"/>
+      <c r="G31" s="153"/>
+      <c r="H31" s="153"/>
+      <c r="I31" s="153"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="130"/>
-      <c r="B32" s="134" t="s">
+      <c r="A32" s="148"/>
+      <c r="B32" s="151" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="135"/>
+      <c r="C32" s="152"/>
       <c r="D32" s="116"/>
       <c r="E32" s="93"/>
       <c r="F32" s="93"/>
-      <c r="G32" s="126"/>
-      <c r="H32" s="126"/>
-      <c r="I32" s="126"/>
+      <c r="G32" s="153"/>
+      <c r="H32" s="153"/>
+      <c r="I32" s="153"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="130"/>
-      <c r="B33" s="134" t="s">
+      <c r="A33" s="148"/>
+      <c r="B33" s="151" t="s">
         <v>44</v>
       </c>
-      <c r="C33" s="135"/>
+      <c r="C33" s="152"/>
       <c r="D33" s="116"/>
       <c r="E33" s="93"/>
       <c r="F33" s="93"/>
-      <c r="G33" s="126"/>
-      <c r="H33" s="126"/>
-      <c r="I33" s="126"/>
+      <c r="G33" s="153"/>
+      <c r="H33" s="153"/>
+      <c r="I33" s="153"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="130"/>
-      <c r="B34" s="134" t="s">
+      <c r="A34" s="148"/>
+      <c r="B34" s="151" t="s">
         <v>45</v>
       </c>
-      <c r="C34" s="135"/>
+      <c r="C34" s="152"/>
       <c r="D34" s="116"/>
       <c r="E34" s="93"/>
       <c r="F34" s="93"/>
-      <c r="G34" s="126"/>
-      <c r="H34" s="126"/>
-      <c r="I34" s="126"/>
+      <c r="G34" s="153"/>
+      <c r="H34" s="153"/>
+      <c r="I34" s="153"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="130"/>
-      <c r="B35" s="134" t="s">
+      <c r="A35" s="148"/>
+      <c r="B35" s="151" t="s">
         <v>46</v>
       </c>
-      <c r="C35" s="135"/>
+      <c r="C35" s="152"/>
       <c r="D35" s="116"/>
       <c r="E35" s="93"/>
       <c r="F35" s="93"/>
-      <c r="G35" s="126"/>
-      <c r="H35" s="126"/>
-      <c r="I35" s="126"/>
+      <c r="G35" s="153"/>
+      <c r="H35" s="153"/>
+      <c r="I35" s="153"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="130"/>
-      <c r="B36" s="134" t="s">
+      <c r="A36" s="148"/>
+      <c r="B36" s="151" t="s">
         <v>47</v>
       </c>
-      <c r="C36" s="135"/>
+      <c r="C36" s="152"/>
       <c r="D36" s="116"/>
       <c r="E36" s="93"/>
       <c r="F36" s="93"/>
-      <c r="G36" s="126"/>
-      <c r="H36" s="126"/>
-      <c r="I36" s="126"/>
+      <c r="G36" s="153"/>
+      <c r="H36" s="153"/>
+      <c r="I36" s="153"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="130"/>
-      <c r="B37" s="134" t="s">
+      <c r="A37" s="148"/>
+      <c r="B37" s="151" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="135"/>
+      <c r="C37" s="152"/>
       <c r="D37" s="116"/>
       <c r="E37" s="93"/>
       <c r="F37" s="93"/>
-      <c r="G37" s="126"/>
-      <c r="H37" s="126"/>
-      <c r="I37" s="126"/>
+      <c r="G37" s="153"/>
+      <c r="H37" s="153"/>
+      <c r="I37" s="153"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="130"/>
-      <c r="B38" s="134" t="s">
+      <c r="A38" s="148"/>
+      <c r="B38" s="151" t="s">
         <v>49</v>
       </c>
-      <c r="C38" s="135"/>
+      <c r="C38" s="152"/>
       <c r="D38" s="116"/>
       <c r="E38" s="93"/>
       <c r="F38" s="93"/>
-      <c r="G38" s="126"/>
-      <c r="H38" s="126"/>
-      <c r="I38" s="126"/>
+      <c r="G38" s="153"/>
+      <c r="H38" s="153"/>
+      <c r="I38" s="153"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="130"/>
-      <c r="B39" s="134" t="s">
+      <c r="A39" s="148"/>
+      <c r="B39" s="151" t="s">
         <v>50</v>
       </c>
-      <c r="C39" s="135"/>
+      <c r="C39" s="152"/>
       <c r="D39" s="116"/>
       <c r="E39" s="93"/>
       <c r="F39" s="93"/>
-      <c r="G39" s="126"/>
-      <c r="H39" s="126"/>
-      <c r="I39" s="126"/>
+      <c r="G39" s="153"/>
+      <c r="H39" s="153"/>
+      <c r="I39" s="153"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="130"/>
-      <c r="B40" s="134" t="s">
+      <c r="A40" s="148"/>
+      <c r="B40" s="151" t="s">
         <v>51</v>
       </c>
-      <c r="C40" s="135"/>
+      <c r="C40" s="152"/>
       <c r="D40" s="116"/>
       <c r="E40" s="93"/>
       <c r="F40" s="93"/>
-      <c r="G40" s="126"/>
-      <c r="H40" s="126"/>
-      <c r="I40" s="126"/>
+      <c r="G40" s="153"/>
+      <c r="H40" s="153"/>
+      <c r="I40" s="153"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="130"/>
-      <c r="B41" s="134" t="s">
+      <c r="A41" s="148"/>
+      <c r="B41" s="151" t="s">
         <v>52</v>
       </c>
-      <c r="C41" s="135"/>
+      <c r="C41" s="152"/>
       <c r="D41" s="116"/>
       <c r="E41" s="93"/>
       <c r="F41" s="93"/>
-      <c r="G41" s="126"/>
-      <c r="H41" s="126"/>
-      <c r="I41" s="126"/>
+      <c r="G41" s="153"/>
+      <c r="H41" s="153"/>
+      <c r="I41" s="153"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="130"/>
-      <c r="B42" s="134" t="s">
+      <c r="A42" s="148"/>
+      <c r="B42" s="151" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="135"/>
+      <c r="C42" s="152"/>
       <c r="D42" s="116"/>
       <c r="E42" s="93"/>
       <c r="F42" s="93"/>
-      <c r="G42" s="126"/>
-      <c r="H42" s="126"/>
-      <c r="I42" s="126"/>
+      <c r="G42" s="153"/>
+      <c r="H42" s="153"/>
+      <c r="I42" s="153"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="130"/>
-      <c r="B43" s="134" t="s">
+      <c r="A43" s="148"/>
+      <c r="B43" s="151" t="s">
         <v>54</v>
       </c>
-      <c r="C43" s="135"/>
+      <c r="C43" s="152"/>
       <c r="D43" s="116"/>
       <c r="E43" s="93"/>
       <c r="F43" s="93"/>
-      <c r="G43" s="126"/>
-      <c r="H43" s="126"/>
-      <c r="I43" s="126"/>
+      <c r="G43" s="153"/>
+      <c r="H43" s="153"/>
+      <c r="I43" s="153"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="130"/>
-      <c r="B44" s="134" t="s">
+      <c r="A44" s="148"/>
+      <c r="B44" s="151" t="s">
         <v>55</v>
       </c>
-      <c r="C44" s="135"/>
+      <c r="C44" s="152"/>
       <c r="D44" s="116"/>
       <c r="E44" s="93"/>
       <c r="F44" s="93"/>
-      <c r="G44" s="126"/>
-      <c r="H44" s="126"/>
-      <c r="I44" s="126"/>
+      <c r="G44" s="153"/>
+      <c r="H44" s="153"/>
+      <c r="I44" s="153"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" s="130"/>
-      <c r="B45" s="134" t="s">
+      <c r="A45" s="148"/>
+      <c r="B45" s="151" t="s">
         <v>56</v>
       </c>
-      <c r="C45" s="135"/>
+      <c r="C45" s="152"/>
       <c r="D45" s="116"/>
       <c r="E45" s="93"/>
       <c r="F45" s="93"/>
-      <c r="G45" s="126"/>
-      <c r="H45" s="126"/>
-      <c r="I45" s="126"/>
+      <c r="G45" s="153"/>
+      <c r="H45" s="153"/>
+      <c r="I45" s="153"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="130"/>
-      <c r="B46" s="134" t="s">
+      <c r="A46" s="148"/>
+      <c r="B46" s="151" t="s">
         <v>57</v>
       </c>
-      <c r="C46" s="135"/>
+      <c r="C46" s="152"/>
       <c r="D46" s="116"/>
       <c r="E46" s="93"/>
       <c r="F46" s="93"/>
-      <c r="G46" s="126"/>
-      <c r="H46" s="126"/>
-      <c r="I46" s="126"/>
+      <c r="G46" s="153"/>
+      <c r="H46" s="153"/>
+      <c r="I46" s="153"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" s="130"/>
-      <c r="B47" s="134" t="s">
+      <c r="A47" s="148"/>
+      <c r="B47" s="151" t="s">
         <v>58</v>
       </c>
-      <c r="C47" s="135"/>
+      <c r="C47" s="152"/>
       <c r="D47" s="116"/>
       <c r="E47" s="93"/>
       <c r="F47" s="93"/>
-      <c r="G47" s="126"/>
-      <c r="H47" s="126"/>
-      <c r="I47" s="126"/>
+      <c r="G47" s="153"/>
+      <c r="H47" s="153"/>
+      <c r="I47" s="153"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A48" s="130"/>
-      <c r="B48" s="132" t="s">
+      <c r="A48" s="148"/>
+      <c r="B48" s="157" t="s">
         <v>59</v>
       </c>
-      <c r="C48" s="133"/>
+      <c r="C48" s="158"/>
       <c r="D48" s="116"/>
       <c r="E48" s="93"/>
       <c r="F48" s="93"/>
-      <c r="G48" s="126"/>
-      <c r="H48" s="126"/>
-      <c r="I48" s="126"/>
+      <c r="G48" s="153"/>
+      <c r="H48" s="153"/>
+      <c r="I48" s="153"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A49" s="130"/>
-      <c r="B49" s="134" t="s">
+      <c r="A49" s="148"/>
+      <c r="B49" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="C49" s="135"/>
+      <c r="C49" s="152"/>
       <c r="D49" s="116"/>
       <c r="E49" s="93"/>
       <c r="F49" s="93"/>
-      <c r="G49" s="126"/>
-      <c r="H49" s="126"/>
-      <c r="I49" s="126"/>
+      <c r="G49" s="153"/>
+      <c r="H49" s="153"/>
+      <c r="I49" s="153"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="117"/>
@@ -6900,65 +6838,65 @@
       <c r="D50" s="118"/>
       <c r="E50" s="111"/>
       <c r="F50" s="119"/>
-      <c r="G50" s="136"/>
-      <c r="H50" s="136"/>
-      <c r="I50" s="136"/>
+      <c r="G50" s="159"/>
+      <c r="H50" s="159"/>
+      <c r="I50" s="159"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A51" s="137" t="s">
+      <c r="A51" s="160" t="s">
         <v>61</v>
       </c>
-      <c r="B51" s="139" t="s">
+      <c r="B51" s="149" t="s">
         <v>62</v>
       </c>
-      <c r="C51" s="140"/>
+      <c r="C51" s="150"/>
       <c r="D51" s="100" t="s">
         <v>63</v>
       </c>
       <c r="E51" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="F51" s="139" t="s">
+      <c r="F51" s="149" t="s">
         <v>38</v>
       </c>
-      <c r="G51" s="141"/>
-      <c r="H51" s="141"/>
-      <c r="I51" s="141"/>
+      <c r="G51" s="162"/>
+      <c r="H51" s="162"/>
+      <c r="I51" s="162"/>
     </row>
     <row r="52" spans="1:10" s="121" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="137"/>
-      <c r="B52" s="127"/>
-      <c r="C52" s="128"/>
+      <c r="A52" s="160"/>
+      <c r="B52" s="163"/>
+      <c r="C52" s="164"/>
       <c r="D52" s="116"/>
       <c r="E52" s="116"/>
-      <c r="F52" s="129"/>
-      <c r="G52" s="129"/>
-      <c r="H52" s="129"/>
-      <c r="I52" s="129"/>
+      <c r="F52" s="165"/>
+      <c r="G52" s="165"/>
+      <c r="H52" s="165"/>
+      <c r="I52" s="165"/>
       <c r="J52" s="120"/>
     </row>
     <row r="53" spans="1:10" s="121" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="137"/>
-      <c r="B53" s="127"/>
-      <c r="C53" s="128"/>
+      <c r="A53" s="160"/>
+      <c r="B53" s="163"/>
+      <c r="C53" s="164"/>
       <c r="D53" s="116"/>
       <c r="E53" s="116"/>
-      <c r="F53" s="129"/>
-      <c r="G53" s="129"/>
-      <c r="H53" s="129"/>
-      <c r="I53" s="129"/>
+      <c r="F53" s="165"/>
+      <c r="G53" s="165"/>
+      <c r="H53" s="165"/>
+      <c r="I53" s="165"/>
       <c r="J53" s="120"/>
     </row>
     <row r="54" spans="1:10" s="121" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="138"/>
-      <c r="B54" s="127"/>
-      <c r="C54" s="128"/>
+      <c r="A54" s="161"/>
+      <c r="B54" s="163"/>
+      <c r="C54" s="164"/>
       <c r="D54" s="116"/>
       <c r="E54" s="116"/>
-      <c r="F54" s="129"/>
-      <c r="G54" s="129"/>
-      <c r="H54" s="129"/>
-      <c r="I54" s="129"/>
+      <c r="F54" s="165"/>
+      <c r="G54" s="165"/>
+      <c r="H54" s="165"/>
+      <c r="I54" s="165"/>
       <c r="J54" s="120"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
@@ -6972,7 +6910,7 @@
       <c r="I55" s="119"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A56" s="130" t="s">
+      <c r="A56" s="148" t="s">
         <v>65</v>
       </c>
       <c r="B56" s="100" t="s">
@@ -6984,93 +6922,93 @@
       <c r="D56" s="100" t="s">
         <v>68</v>
       </c>
-      <c r="E56" s="131" t="s">
+      <c r="E56" s="166" t="s">
         <v>38</v>
       </c>
-      <c r="F56" s="131"/>
-      <c r="G56" s="131"/>
-      <c r="H56" s="131"/>
-      <c r="I56" s="131"/>
+      <c r="F56" s="166"/>
+      <c r="G56" s="166"/>
+      <c r="H56" s="166"/>
+      <c r="I56" s="166"/>
       <c r="J56" s="91" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A57" s="130"/>
+      <c r="A57" s="148"/>
       <c r="B57" s="122" t="s">
         <v>70</v>
       </c>
       <c r="C57" s="123"/>
       <c r="D57" s="39"/>
-      <c r="E57" s="126"/>
-      <c r="F57" s="126"/>
-      <c r="G57" s="126"/>
-      <c r="H57" s="126"/>
-      <c r="I57" s="126"/>
+      <c r="E57" s="153"/>
+      <c r="F57" s="153"/>
+      <c r="G57" s="153"/>
+      <c r="H57" s="153"/>
+      <c r="I57" s="153"/>
       <c r="J57" s="91" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A58" s="130"/>
+      <c r="A58" s="148"/>
       <c r="B58" s="122" t="s">
         <v>71</v>
       </c>
       <c r="C58" s="123"/>
       <c r="D58" s="123"/>
-      <c r="E58" s="126"/>
-      <c r="F58" s="126"/>
-      <c r="G58" s="126"/>
-      <c r="H58" s="126"/>
-      <c r="I58" s="126"/>
+      <c r="E58" s="153"/>
+      <c r="F58" s="153"/>
+      <c r="G58" s="153"/>
+      <c r="H58" s="153"/>
+      <c r="I58" s="153"/>
       <c r="J58" s="91" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A59" s="130"/>
+      <c r="A59" s="148"/>
       <c r="B59" s="122" t="s">
         <v>69</v>
       </c>
       <c r="C59" s="123"/>
       <c r="D59" s="123"/>
-      <c r="E59" s="126"/>
-      <c r="F59" s="126"/>
-      <c r="G59" s="126"/>
-      <c r="H59" s="126"/>
-      <c r="I59" s="126"/>
+      <c r="E59" s="153"/>
+      <c r="F59" s="153"/>
+      <c r="G59" s="153"/>
+      <c r="H59" s="153"/>
+      <c r="I59" s="153"/>
       <c r="J59" s="91" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A60" s="130"/>
+      <c r="A60" s="148"/>
       <c r="B60" s="122" t="s">
         <v>69</v>
       </c>
       <c r="C60" s="123"/>
       <c r="D60" s="123"/>
-      <c r="E60" s="126"/>
-      <c r="F60" s="126"/>
-      <c r="G60" s="126"/>
-      <c r="H60" s="126"/>
-      <c r="I60" s="126"/>
+      <c r="E60" s="153"/>
+      <c r="F60" s="153"/>
+      <c r="G60" s="153"/>
+      <c r="H60" s="153"/>
+      <c r="I60" s="153"/>
       <c r="J60" s="91" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A61" s="130"/>
+      <c r="A61" s="148"/>
       <c r="B61" s="122" t="s">
         <v>69</v>
       </c>
       <c r="C61" s="123"/>
       <c r="D61" s="39"/>
-      <c r="E61" s="126"/>
-      <c r="F61" s="126"/>
-      <c r="G61" s="126"/>
-      <c r="H61" s="126"/>
-      <c r="I61" s="126"/>
+      <c r="E61" s="153"/>
+      <c r="F61" s="153"/>
+      <c r="G61" s="153"/>
+      <c r="H61" s="153"/>
+      <c r="I61" s="153"/>
       <c r="J61" s="91" t="s">
         <v>74</v>
       </c>
@@ -7251,43 +7189,50 @@
     </row>
   </sheetData>
   <mergeCells count="105">
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="A5:A9"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="B10:I10"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="E61:I61"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="F54:I54"/>
+    <mergeCell ref="A56:A61"/>
+    <mergeCell ref="E56:I56"/>
+    <mergeCell ref="E57:I57"/>
+    <mergeCell ref="E58:I58"/>
+    <mergeCell ref="E59:I59"/>
+    <mergeCell ref="E60:I60"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="F52:I52"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="G39:I39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="G38:I38"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="G25:I25"/>
@@ -7312,50 +7257,43 @@
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="G32:I32"/>
     <mergeCell ref="B39:C39"/>
-    <mergeCell ref="G39:I39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="G41:I41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="G38:I38"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="G46:I46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:I51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="F52:I52"/>
-    <mergeCell ref="E61:I61"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="A56:A61"/>
-    <mergeCell ref="E56:I56"/>
-    <mergeCell ref="E57:I57"/>
-    <mergeCell ref="E58:I58"/>
-    <mergeCell ref="E59:I59"/>
-    <mergeCell ref="E60:I60"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="B10:I10"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="A5:A9"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="G18:I18"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B57:B61" xr:uid="{DE5F0C72-FF19-4C19-9AAC-1DA4927D9237}">
@@ -8630,29 +8568,29 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="175">
+      <c r="A2" s="174">
         <v>1</v>
       </c>
-      <c r="B2" s="178"/>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="179"/>
-      <c r="L2" s="179"/>
-      <c r="M2" s="179"/>
-      <c r="N2" s="179"/>
-      <c r="O2" s="180"/>
+      <c r="B2" s="177"/>
+      <c r="C2" s="178"/>
+      <c r="D2" s="178"/>
+      <c r="E2" s="178"/>
+      <c r="F2" s="178"/>
+      <c r="G2" s="178"/>
+      <c r="H2" s="178"/>
+      <c r="I2" s="178"/>
+      <c r="J2" s="178"/>
+      <c r="K2" s="178"/>
+      <c r="L2" s="178"/>
+      <c r="M2" s="178"/>
+      <c r="N2" s="178"/>
+      <c r="O2" s="179"/>
     </row>
     <row r="3" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="176"/>
-      <c r="B3" s="181"/>
-      <c r="C3" s="184"/>
-      <c r="D3" s="187"/>
+      <c r="A3" s="175"/>
+      <c r="B3" s="180"/>
+      <c r="C3" s="183"/>
+      <c r="D3" s="186"/>
       <c r="E3" s="46" t="s">
         <v>412</v>
       </c>
@@ -8674,10 +8612,10 @@
       <c r="O3" s="52"/>
     </row>
     <row r="4" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="176"/>
-      <c r="B4" s="182"/>
-      <c r="C4" s="185"/>
-      <c r="D4" s="188"/>
+      <c r="A4" s="175"/>
+      <c r="B4" s="181"/>
+      <c r="C4" s="184"/>
+      <c r="D4" s="187"/>
       <c r="E4" s="46" t="s">
         <v>416</v>
       </c>
@@ -8699,10 +8637,10 @@
       <c r="O4" s="52"/>
     </row>
     <row r="5" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A5" s="176"/>
-      <c r="B5" s="182"/>
-      <c r="C5" s="185"/>
-      <c r="D5" s="188"/>
+      <c r="A5" s="175"/>
+      <c r="B5" s="181"/>
+      <c r="C5" s="184"/>
+      <c r="D5" s="187"/>
       <c r="E5" s="46" t="s">
         <v>418</v>
       </c>
@@ -8724,10 +8662,10 @@
       <c r="O5" s="52"/>
     </row>
     <row r="6" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A6" s="176"/>
-      <c r="B6" s="182"/>
-      <c r="C6" s="185"/>
-      <c r="D6" s="188"/>
+      <c r="A6" s="175"/>
+      <c r="B6" s="181"/>
+      <c r="C6" s="184"/>
+      <c r="D6" s="187"/>
       <c r="E6" s="46" t="s">
         <v>419</v>
       </c>
@@ -8749,10 +8687,10 @@
       <c r="O6" s="52"/>
     </row>
     <row r="7" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A7" s="176"/>
-      <c r="B7" s="182"/>
-      <c r="C7" s="185"/>
-      <c r="D7" s="188"/>
+      <c r="A7" s="175"/>
+      <c r="B7" s="181"/>
+      <c r="C7" s="184"/>
+      <c r="D7" s="187"/>
       <c r="E7" s="46" t="s">
         <v>420</v>
       </c>
@@ -8774,10 +8712,10 @@
       <c r="O7" s="52"/>
     </row>
     <row r="8" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A8" s="176"/>
-      <c r="B8" s="182"/>
-      <c r="C8" s="185"/>
-      <c r="D8" s="188"/>
+      <c r="A8" s="175"/>
+      <c r="B8" s="181"/>
+      <c r="C8" s="184"/>
+      <c r="D8" s="187"/>
       <c r="E8" s="46" t="s">
         <v>421</v>
       </c>
@@ -8799,10 +8737,10 @@
       <c r="O8" s="52"/>
     </row>
     <row r="9" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A9" s="176"/>
-      <c r="B9" s="182"/>
-      <c r="C9" s="185"/>
-      <c r="D9" s="188"/>
+      <c r="A9" s="175"/>
+      <c r="B9" s="181"/>
+      <c r="C9" s="184"/>
+      <c r="D9" s="187"/>
       <c r="E9" s="46" t="s">
         <v>422</v>
       </c>
@@ -8824,10 +8762,10 @@
       <c r="O9" s="52"/>
     </row>
     <row r="10" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A10" s="176"/>
-      <c r="B10" s="182"/>
-      <c r="C10" s="185"/>
-      <c r="D10" s="188"/>
+      <c r="A10" s="175"/>
+      <c r="B10" s="181"/>
+      <c r="C10" s="184"/>
+      <c r="D10" s="187"/>
       <c r="E10" s="46" t="s">
         <v>423</v>
       </c>
@@ -8849,10 +8787,10 @@
       <c r="O10" s="52"/>
     </row>
     <row r="11" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A11" s="176"/>
-      <c r="B11" s="182"/>
-      <c r="C11" s="185"/>
-      <c r="D11" s="188"/>
+      <c r="A11" s="175"/>
+      <c r="B11" s="181"/>
+      <c r="C11" s="184"/>
+      <c r="D11" s="187"/>
       <c r="E11" s="46" t="s">
         <v>424</v>
       </c>
@@ -8874,10 +8812,10 @@
       <c r="O11" s="52"/>
     </row>
     <row r="12" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A12" s="176"/>
-      <c r="B12" s="182"/>
-      <c r="C12" s="185"/>
-      <c r="D12" s="188"/>
+      <c r="A12" s="175"/>
+      <c r="B12" s="181"/>
+      <c r="C12" s="184"/>
+      <c r="D12" s="187"/>
       <c r="E12" s="46" t="s">
         <v>425</v>
       </c>
@@ -8899,10 +8837,10 @@
       <c r="O12" s="52"/>
     </row>
     <row r="13" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A13" s="176"/>
-      <c r="B13" s="182"/>
-      <c r="C13" s="185"/>
-      <c r="D13" s="188"/>
+      <c r="A13" s="175"/>
+      <c r="B13" s="181"/>
+      <c r="C13" s="184"/>
+      <c r="D13" s="187"/>
       <c r="E13" s="46" t="s">
         <v>426</v>
       </c>
@@ -8924,10 +8862,10 @@
       <c r="O13" s="52"/>
     </row>
     <row r="14" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A14" s="176"/>
-      <c r="B14" s="182"/>
-      <c r="C14" s="185"/>
-      <c r="D14" s="188"/>
+      <c r="A14" s="175"/>
+      <c r="B14" s="181"/>
+      <c r="C14" s="184"/>
+      <c r="D14" s="187"/>
       <c r="E14" s="46" t="s">
         <v>427</v>
       </c>
@@ -8949,10 +8887,10 @@
       <c r="O14" s="52"/>
     </row>
     <row r="15" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A15" s="176"/>
-      <c r="B15" s="182"/>
-      <c r="C15" s="185"/>
-      <c r="D15" s="188"/>
+      <c r="A15" s="175"/>
+      <c r="B15" s="181"/>
+      <c r="C15" s="184"/>
+      <c r="D15" s="187"/>
       <c r="E15" s="46" t="s">
         <v>428</v>
       </c>
@@ -8974,10 +8912,10 @@
       <c r="O15" s="52"/>
     </row>
     <row r="16" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A16" s="176"/>
-      <c r="B16" s="182"/>
-      <c r="C16" s="185"/>
-      <c r="D16" s="188"/>
+      <c r="A16" s="175"/>
+      <c r="B16" s="181"/>
+      <c r="C16" s="184"/>
+      <c r="D16" s="187"/>
       <c r="E16" s="46" t="s">
         <v>429</v>
       </c>
@@ -8999,10 +8937,10 @@
       <c r="O16" s="52"/>
     </row>
     <row r="17" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A17" s="176"/>
-      <c r="B17" s="182"/>
-      <c r="C17" s="185"/>
-      <c r="D17" s="188"/>
+      <c r="A17" s="175"/>
+      <c r="B17" s="181"/>
+      <c r="C17" s="184"/>
+      <c r="D17" s="187"/>
       <c r="E17" s="46" t="s">
         <v>430</v>
       </c>
@@ -9024,10 +8962,10 @@
       <c r="O17" s="52"/>
     </row>
     <row r="18" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A18" s="176"/>
-      <c r="B18" s="182"/>
-      <c r="C18" s="185"/>
-      <c r="D18" s="188"/>
+      <c r="A18" s="175"/>
+      <c r="B18" s="181"/>
+      <c r="C18" s="184"/>
+      <c r="D18" s="187"/>
       <c r="E18" s="46" t="s">
         <v>431</v>
       </c>
@@ -9049,10 +8987,10 @@
       <c r="O18" s="52"/>
     </row>
     <row r="19" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A19" s="176"/>
-      <c r="B19" s="182"/>
-      <c r="C19" s="185"/>
-      <c r="D19" s="188"/>
+      <c r="A19" s="175"/>
+      <c r="B19" s="181"/>
+      <c r="C19" s="184"/>
+      <c r="D19" s="187"/>
       <c r="E19" s="46" t="s">
         <v>432</v>
       </c>
@@ -9074,10 +9012,10 @@
       <c r="O19" s="52"/>
     </row>
     <row r="20" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A20" s="176"/>
-      <c r="B20" s="182"/>
-      <c r="C20" s="185"/>
-      <c r="D20" s="188"/>
+      <c r="A20" s="175"/>
+      <c r="B20" s="181"/>
+      <c r="C20" s="184"/>
+      <c r="D20" s="187"/>
       <c r="E20" s="53" t="s">
         <v>433</v>
       </c>
@@ -9099,10 +9037,10 @@
       <c r="O20" s="58"/>
     </row>
     <row r="21" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A21" s="176"/>
-      <c r="B21" s="182"/>
-      <c r="C21" s="185"/>
-      <c r="D21" s="188"/>
+      <c r="A21" s="175"/>
+      <c r="B21" s="181"/>
+      <c r="C21" s="184"/>
+      <c r="D21" s="187"/>
       <c r="E21" s="53" t="s">
         <v>434</v>
       </c>
@@ -9124,10 +9062,10 @@
       <c r="O21" s="58"/>
     </row>
     <row r="22" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A22" s="176"/>
-      <c r="B22" s="182"/>
-      <c r="C22" s="185"/>
-      <c r="D22" s="188"/>
+      <c r="A22" s="175"/>
+      <c r="B22" s="181"/>
+      <c r="C22" s="184"/>
+      <c r="D22" s="187"/>
       <c r="E22" s="46" t="s">
         <v>435</v>
       </c>
@@ -9147,10 +9085,10 @@
       <c r="O22" s="52"/>
     </row>
     <row r="23" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A23" s="176"/>
-      <c r="B23" s="182"/>
-      <c r="C23" s="185"/>
-      <c r="D23" s="188"/>
+      <c r="A23" s="175"/>
+      <c r="B23" s="181"/>
+      <c r="C23" s="184"/>
+      <c r="D23" s="187"/>
       <c r="E23" s="46" t="s">
         <v>437</v>
       </c>
@@ -9170,10 +9108,10 @@
       <c r="O23" s="52"/>
     </row>
     <row r="24" spans="1:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="A24" s="176"/>
-      <c r="B24" s="182"/>
-      <c r="C24" s="185"/>
-      <c r="D24" s="188"/>
+      <c r="A24" s="175"/>
+      <c r="B24" s="181"/>
+      <c r="C24" s="184"/>
+      <c r="D24" s="187"/>
       <c r="E24" s="46" t="s">
         <v>438</v>
       </c>
@@ -9193,10 +9131,10 @@
       <c r="O24" s="52"/>
     </row>
     <row r="25" spans="1:15" ht="21" x14ac:dyDescent="0.3">
-      <c r="A25" s="176"/>
-      <c r="B25" s="182"/>
-      <c r="C25" s="185"/>
-      <c r="D25" s="188"/>
+      <c r="A25" s="175"/>
+      <c r="B25" s="181"/>
+      <c r="C25" s="184"/>
+      <c r="D25" s="187"/>
       <c r="E25" s="46" t="s">
         <v>439</v>
       </c>
@@ -9226,10 +9164,10 @@
       <c r="O25" s="52"/>
     </row>
     <row r="26" spans="1:15" ht="21" x14ac:dyDescent="0.3">
-      <c r="A26" s="176"/>
-      <c r="B26" s="182"/>
-      <c r="C26" s="185"/>
-      <c r="D26" s="188"/>
+      <c r="A26" s="175"/>
+      <c r="B26" s="181"/>
+      <c r="C26" s="184"/>
+      <c r="D26" s="187"/>
       <c r="E26" s="46" t="s">
         <v>442</v>
       </c>
@@ -9259,10 +9197,10 @@
       <c r="O26" s="52"/>
     </row>
     <row r="27" spans="1:15" ht="21" x14ac:dyDescent="0.3">
-      <c r="A27" s="176"/>
-      <c r="B27" s="182"/>
-      <c r="C27" s="185"/>
-      <c r="D27" s="188"/>
+      <c r="A27" s="175"/>
+      <c r="B27" s="181"/>
+      <c r="C27" s="184"/>
+      <c r="D27" s="187"/>
       <c r="E27" s="46" t="s">
         <v>443</v>
       </c>
@@ -9282,10 +9220,10 @@
       <c r="O27" s="52"/>
     </row>
     <row r="28" spans="1:15" ht="21" x14ac:dyDescent="0.3">
-      <c r="A28" s="176"/>
-      <c r="B28" s="182"/>
-      <c r="C28" s="185"/>
-      <c r="D28" s="188"/>
+      <c r="A28" s="175"/>
+      <c r="B28" s="181"/>
+      <c r="C28" s="184"/>
+      <c r="D28" s="187"/>
       <c r="E28" s="46" t="s">
         <v>445</v>
       </c>
@@ -9305,10 +9243,10 @@
       <c r="O28" s="52"/>
     </row>
     <row r="29" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A29" s="176"/>
-      <c r="B29" s="182"/>
-      <c r="C29" s="185"/>
-      <c r="D29" s="188"/>
+      <c r="A29" s="175"/>
+      <c r="B29" s="181"/>
+      <c r="C29" s="184"/>
+      <c r="D29" s="187"/>
       <c r="E29" s="46" t="s">
         <v>446</v>
       </c>
@@ -9330,10 +9268,10 @@
       <c r="O29" s="52"/>
     </row>
     <row r="30" spans="1:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="177"/>
-      <c r="B30" s="183"/>
-      <c r="C30" s="186"/>
-      <c r="D30" s="189"/>
+      <c r="A30" s="176"/>
+      <c r="B30" s="182"/>
+      <c r="C30" s="185"/>
+      <c r="D30" s="188"/>
       <c r="E30" s="66" t="s">
         <v>448</v>
       </c>
@@ -10688,10 +10626,10 @@
   <sheetData>
     <row r="1" spans="2:3" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="167" t="s">
         <v>92</v>
       </c>
-      <c r="C2" s="169"/>
+      <c r="C2" s="168"/>
     </row>
     <row r="3" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
@@ -10835,10 +10773,10 @@
     </row>
     <row r="24" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="25" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="168" t="s">
+      <c r="B25" s="167" t="s">
         <v>121</v>
       </c>
-      <c r="C25" s="169"/>
+      <c r="C25" s="168"/>
       <c r="E25" s="74" t="s">
         <v>122</v>
       </c>
@@ -10929,10 +10867,10 @@
     </row>
     <row r="40" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="41" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="170" t="s">
+      <c r="B41" s="169" t="s">
         <v>128</v>
       </c>
-      <c r="C41" s="171"/>
+      <c r="C41" s="170"/>
     </row>
     <row r="42" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B42" s="5" t="s">
@@ -11002,10 +10940,10 @@
     </row>
     <row r="53" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="54" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="170" t="s">
+      <c r="B54" s="169" t="s">
         <v>140</v>
       </c>
-      <c r="C54" s="171"/>
+      <c r="C54" s="170"/>
     </row>
     <row r="55" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B55" s="5" t="s">
@@ -11039,10 +10977,10 @@
     </row>
     <row r="60" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="61" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="168" t="s">
+      <c r="B61" s="167" t="s">
         <v>146</v>
       </c>
-      <c r="C61" s="169"/>
+      <c r="C61" s="168"/>
     </row>
     <row r="62" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B62" s="5" t="s">
@@ -11054,10 +10992,10 @@
       <c r="C63" s="15"/>
     </row>
     <row r="64" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B64" s="170" t="s">
+      <c r="B64" s="169" t="s">
         <v>148</v>
       </c>
-      <c r="C64" s="171"/>
+      <c r="C64" s="170"/>
     </row>
     <row r="65" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B65" s="5" t="s">
@@ -11085,10 +11023,10 @@
     </row>
     <row r="69" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="70" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B70" s="168" t="s">
+      <c r="B70" s="167" t="s">
         <v>153</v>
       </c>
-      <c r="C70" s="169"/>
+      <c r="C70" s="168"/>
     </row>
     <row r="71" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B71" s="5"/>
@@ -11132,10 +11070,10 @@
     </row>
     <row r="81" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="82" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B82" s="168" t="s">
+      <c r="B82" s="167" t="s">
         <v>154</v>
       </c>
-      <c r="C82" s="169"/>
+      <c r="C82" s="168"/>
     </row>
     <row r="83" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B83" s="5"/>
@@ -11179,10 +11117,10 @@
     </row>
     <row r="93" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="94" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B94" s="168" t="s">
+      <c r="B94" s="167" t="s">
         <v>155</v>
       </c>
-      <c r="C94" s="169"/>
+      <c r="C94" s="168"/>
     </row>
     <row r="95" spans="2:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B95" s="5"/>
@@ -11260,19 +11198,19 @@
       <c r="B1" s="12" t="s">
         <v>561</v>
       </c>
-      <c r="C1" s="125" t="s">
+      <c r="C1" s="12" t="s">
         <v>562</v>
       </c>
-      <c r="D1" s="125" t="s">
+      <c r="D1" s="12" t="s">
         <v>581</v>
       </c>
-      <c r="E1" s="125" t="s">
+      <c r="E1" s="12" t="s">
         <v>596</v>
       </c>
-      <c r="F1" s="125" t="s">
+      <c r="F1" s="12" t="s">
         <v>610</v>
       </c>
-      <c r="G1" s="192" t="s">
+      <c r="G1" s="12" t="s">
         <v>614</v>
       </c>
     </row>
@@ -11280,7 +11218,7 @@
       <c r="A2" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="G2" s="190" t="s">
+      <c r="G2" t="s">
         <v>89</v>
       </c>
     </row>
@@ -11301,7 +11239,7 @@
       <c r="F3" s="15" t="s">
         <v>563</v>
       </c>
-      <c r="G3" s="191" t="s">
+      <c r="G3" s="15" t="s">
         <v>615</v>
       </c>
     </row>
@@ -11322,7 +11260,7 @@
       <c r="F4" s="15" t="s">
         <v>564</v>
       </c>
-      <c r="G4" s="191" t="s">
+      <c r="G4" s="15" t="s">
         <v>616</v>
       </c>
     </row>
@@ -11343,7 +11281,7 @@
       <c r="F5" s="15" t="s">
         <v>582</v>
       </c>
-      <c r="G5" s="191" t="s">
+      <c r="G5" s="15" t="s">
         <v>617</v>
       </c>
     </row>
@@ -11356,7 +11294,7 @@
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
-      <c r="G6" s="191"/>
+      <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
@@ -11375,7 +11313,7 @@
       <c r="F7" s="15" t="s">
         <v>611</v>
       </c>
-      <c r="G7" s="191"/>
+      <c r="G7" s="15"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
@@ -11386,7 +11324,7 @@
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
       <c r="F8" s="15"/>
-      <c r="G8" s="191" t="s">
+      <c r="G8" s="15" t="s">
         <v>618</v>
       </c>
     </row>
@@ -11407,7 +11345,7 @@
       <c r="F9" s="15" t="s">
         <v>612</v>
       </c>
-      <c r="G9" s="191" t="s">
+      <c r="G9" s="15" t="s">
         <v>619</v>
       </c>
     </row>
@@ -11428,7 +11366,7 @@
       <c r="F10" s="15" t="s">
         <v>585</v>
       </c>
-      <c r="G10" s="191"/>
+      <c r="G10" s="15"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
@@ -11447,7 +11385,7 @@
       <c r="F11" s="15" t="s">
         <v>586</v>
       </c>
-      <c r="G11" s="191" t="s">
+      <c r="G11" s="15" t="s">
         <v>620</v>
       </c>
     </row>
@@ -11468,7 +11406,7 @@
       <c r="F12" s="15" t="s">
         <v>587</v>
       </c>
-      <c r="G12" s="191" t="s">
+      <c r="G12" s="15" t="s">
         <v>621</v>
       </c>
     </row>
@@ -11489,7 +11427,7 @@
       <c r="F13" s="15" t="s">
         <v>588</v>
       </c>
-      <c r="G13" s="191" t="s">
+      <c r="G13" s="15" t="s">
         <v>622</v>
       </c>
     </row>
@@ -11502,7 +11440,7 @@
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
-      <c r="G14" s="191"/>
+      <c r="G14" s="15"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
@@ -11521,7 +11459,7 @@
       <c r="F15" s="15" t="s">
         <v>572</v>
       </c>
-      <c r="G15" s="191" t="s">
+      <c r="G15" s="15" t="s">
         <v>623</v>
       </c>
     </row>
@@ -11540,7 +11478,7 @@
       <c r="F16" s="15" t="s">
         <v>589</v>
       </c>
-      <c r="G16" s="191" t="s">
+      <c r="G16" s="15" t="s">
         <v>624</v>
       </c>
     </row>
@@ -11557,18 +11495,18 @@
       <c r="F17" s="15" t="s">
         <v>590</v>
       </c>
-      <c r="G17" s="191" t="s">
+      <c r="G17" s="15" t="s">
         <v>624</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="13"/>
       <c r="B18" s="89"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="191"/>
+      <c r="C18" s="89"/>
+      <c r="D18" s="89"/>
+      <c r="E18" s="89"/>
+      <c r="F18" s="89"/>
+      <c r="G18" s="89"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
@@ -11587,7 +11525,7 @@
       <c r="F19" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="G19" s="191" t="s">
+      <c r="G19" s="15" t="s">
         <v>625</v>
       </c>
     </row>
@@ -11604,7 +11542,7 @@
         <v>574</v>
       </c>
       <c r="F20" s="15"/>
-      <c r="G20" s="191"/>
+      <c r="G20" s="15"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
@@ -11621,7 +11559,7 @@
       <c r="F21" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="G21" s="191"/>
+      <c r="G21" s="15"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
@@ -11634,7 +11572,7 @@
         <v>604</v>
       </c>
       <c r="F22" s="15"/>
-      <c r="G22" s="191"/>
+      <c r="G22" s="15"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
@@ -11653,7 +11591,7 @@
       <c r="F23" s="15" t="s">
         <v>592</v>
       </c>
-      <c r="G23" s="191" t="s">
+      <c r="G23" s="15" t="s">
         <v>626</v>
       </c>
     </row>
@@ -11672,7 +11610,7 @@
       <c r="F24" s="15" t="s">
         <v>592</v>
       </c>
-      <c r="G24" s="191" t="s">
+      <c r="G24" s="15" t="s">
         <v>627</v>
       </c>
     </row>
@@ -11685,7 +11623,7 @@
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
       <c r="F25" s="15"/>
-      <c r="G25" s="191" t="s">
+      <c r="G25" s="15" t="s">
         <v>626</v>
       </c>
     </row>
@@ -11698,7 +11636,7 @@
       <c r="D26" s="15"/>
       <c r="E26" s="15"/>
       <c r="F26" s="15"/>
-      <c r="G26" s="191"/>
+      <c r="G26" s="15"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
@@ -11709,7 +11647,7 @@
       <c r="D27" s="15"/>
       <c r="E27" s="15"/>
       <c r="F27" s="15"/>
-      <c r="G27" s="191"/>
+      <c r="G27" s="15"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
@@ -11720,7 +11658,7 @@
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
-      <c r="G28" s="191"/>
+      <c r="G28" s="15"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="13" t="s">
@@ -11731,7 +11669,7 @@
       <c r="D29" s="15"/>
       <c r="E29" s="15"/>
       <c r="F29" s="15"/>
-      <c r="G29" s="191"/>
+      <c r="G29" s="15"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="13" t="s">
@@ -11742,7 +11680,7 @@
       <c r="D30" s="15"/>
       <c r="E30" s="15"/>
       <c r="F30" s="15"/>
-      <c r="G30" s="191"/>
+      <c r="G30" s="15"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
@@ -11753,7 +11691,7 @@
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
       <c r="F31" s="15"/>
-      <c r="G31" s="191"/>
+      <c r="G31" s="15"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="13" t="s">
@@ -11764,7 +11702,7 @@
       <c r="D32" s="15"/>
       <c r="E32" s="15"/>
       <c r="F32" s="15"/>
-      <c r="G32" s="191"/>
+      <c r="G32" s="15"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="13" t="s">
@@ -11775,7 +11713,7 @@
       <c r="D33" s="15"/>
       <c r="E33" s="15"/>
       <c r="F33" s="15"/>
-      <c r="G33" s="191"/>
+      <c r="G33" s="15"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="13" t="s">
@@ -11786,7 +11724,7 @@
       <c r="D34" s="15"/>
       <c r="E34" s="15"/>
       <c r="F34" s="15"/>
-      <c r="G34" s="191"/>
+      <c r="G34" s="15"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="13" t="s">
@@ -11797,7 +11735,7 @@
       <c r="D35" s="15"/>
       <c r="E35" s="15"/>
       <c r="F35" s="15"/>
-      <c r="G35" s="191"/>
+      <c r="G35" s="15"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="13" t="s">
@@ -11808,7 +11746,7 @@
       <c r="D36" s="15"/>
       <c r="E36" s="15"/>
       <c r="F36" s="15"/>
-      <c r="G36" s="191"/>
+      <c r="G36" s="15"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="14" t="s">
@@ -11819,7 +11757,7 @@
       <c r="D37" s="15"/>
       <c r="E37" s="15"/>
       <c r="F37" s="15"/>
-      <c r="G37" s="191"/>
+      <c r="G37" s="15"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="14" t="s">
@@ -11830,7 +11768,7 @@
       <c r="D38" s="15"/>
       <c r="E38" s="15"/>
       <c r="F38" s="15"/>
-      <c r="G38" s="191"/>
+      <c r="G38" s="15"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
@@ -11841,7 +11779,7 @@
       <c r="D39" s="15"/>
       <c r="E39" s="15"/>
       <c r="F39" s="15"/>
-      <c r="G39" s="191"/>
+      <c r="G39" s="15"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
@@ -11852,7 +11790,7 @@
       <c r="D40" s="15"/>
       <c r="E40" s="15"/>
       <c r="F40" s="15"/>
-      <c r="G40" s="191"/>
+      <c r="G40" s="15"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
@@ -11863,16 +11801,16 @@
       <c r="D41" s="15"/>
       <c r="E41" s="15"/>
       <c r="F41" s="15"/>
-      <c r="G41" s="191"/>
+      <c r="G41" s="15"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="13"/>
       <c r="B42" s="89"/>
-      <c r="C42" s="15"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="191"/>
+      <c r="C42" s="89"/>
+      <c r="D42" s="89"/>
+      <c r="E42" s="89"/>
+      <c r="F42" s="89"/>
+      <c r="G42" s="89"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
@@ -11883,7 +11821,7 @@
       <c r="D43" s="15"/>
       <c r="E43" s="15"/>
       <c r="F43" s="15"/>
-      <c r="G43" s="191" t="s">
+      <c r="G43" s="15" t="s">
         <v>628</v>
       </c>
     </row>
@@ -11904,7 +11842,7 @@
       <c r="F44" s="15" t="s">
         <v>593</v>
       </c>
-      <c r="G44" s="191"/>
+      <c r="G44" s="15"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="13" t="s">
@@ -11923,7 +11861,7 @@
       <c r="F45" s="15" t="s">
         <v>613</v>
       </c>
-      <c r="G45" s="191" t="s">
+      <c r="G45" s="15" t="s">
         <v>629</v>
       </c>
     </row>
@@ -11940,7 +11878,7 @@
       </c>
       <c r="E46" s="15"/>
       <c r="F46" s="15"/>
-      <c r="G46" s="191" t="s">
+      <c r="G46" s="15" t="s">
         <v>630</v>
       </c>
     </row>
@@ -11957,7 +11895,7 @@
       </c>
       <c r="E47" s="15"/>
       <c r="F47" s="15"/>
-      <c r="G47" s="191" t="s">
+      <c r="G47" s="15" t="s">
         <v>413</v>
       </c>
     </row>
@@ -11970,7 +11908,7 @@
       <c r="D48" s="15"/>
       <c r="E48" s="15"/>
       <c r="F48" s="15"/>
-      <c r="G48" s="191" t="s">
+      <c r="G48" s="15" t="s">
         <v>631</v>
       </c>
     </row>
@@ -11983,7 +11921,7 @@
       <c r="D49" s="15"/>
       <c r="E49" s="15"/>
       <c r="F49" s="15"/>
-      <c r="G49" s="191" t="s">
+      <c r="G49" s="15" t="s">
         <v>632</v>
       </c>
     </row>
@@ -12000,7 +11938,7 @@
         <v>579</v>
       </c>
       <c r="F50" s="15"/>
-      <c r="G50" s="191"/>
+      <c r="G50" s="15"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="13" t="s">
@@ -12015,7 +11953,7 @@
         <v>608</v>
       </c>
       <c r="F51" s="15"/>
-      <c r="G51" s="191" t="s">
+      <c r="G51" s="15" t="s">
         <v>633</v>
       </c>
     </row>
@@ -12030,7 +11968,7 @@
         <v>609</v>
       </c>
       <c r="F52" s="15"/>
-      <c r="G52" s="191" t="s">
+      <c r="G52" s="15" t="s">
         <v>634</v>
       </c>
     </row>
@@ -12043,7 +11981,7 @@
       <c r="D53" s="15"/>
       <c r="E53" s="15"/>
       <c r="F53" s="15"/>
-      <c r="G53" s="191" t="s">
+      <c r="G53" s="15" t="s">
         <v>413</v>
       </c>
     </row>
@@ -12056,7 +11994,7 @@
       <c r="D54" s="15"/>
       <c r="E54" s="15"/>
       <c r="F54" s="15"/>
-      <c r="G54" s="191"/>
+      <c r="G54" s="15"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
@@ -12067,7 +12005,7 @@
       <c r="D55" s="15"/>
       <c r="E55" s="15"/>
       <c r="F55" s="15"/>
-      <c r="G55" s="191" t="s">
+      <c r="G55" s="15" t="s">
         <v>635</v>
       </c>
     </row>
@@ -12080,7 +12018,7 @@
       <c r="D56" s="15"/>
       <c r="E56" s="15"/>
       <c r="F56" s="15"/>
-      <c r="G56" s="191"/>
+      <c r="G56" s="15"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="13" t="s">
@@ -12091,7 +12029,7 @@
       <c r="D57" s="15"/>
       <c r="E57" s="15"/>
       <c r="F57" s="15"/>
-      <c r="G57" s="191" t="s">
+      <c r="G57" s="15" t="s">
         <v>636</v>
       </c>
     </row>
@@ -12104,7 +12042,7 @@
       <c r="D58" s="15"/>
       <c r="E58" s="15"/>
       <c r="F58" s="15"/>
-      <c r="G58" s="191" t="s">
+      <c r="G58" s="15" t="s">
         <v>637</v>
       </c>
     </row>
@@ -12117,7 +12055,7 @@
       <c r="D59" s="15"/>
       <c r="E59" s="15"/>
       <c r="F59" s="15"/>
-      <c r="G59" s="191" t="s">
+      <c r="G59" s="15" t="s">
         <v>638</v>
       </c>
     </row>
@@ -12130,7 +12068,7 @@
       <c r="D60" s="15"/>
       <c r="E60" s="15"/>
       <c r="F60" s="15"/>
-      <c r="G60" s="191" t="s">
+      <c r="G60" s="15" t="s">
         <v>639</v>
       </c>
     </row>
@@ -12143,7 +12081,7 @@
       <c r="D61" s="15"/>
       <c r="E61" s="15"/>
       <c r="F61" s="15"/>
-      <c r="G61" s="191" t="s">
+      <c r="G61" s="15" t="s">
         <v>640</v>
       </c>
     </row>
@@ -12156,7 +12094,7 @@
       <c r="D62" s="15"/>
       <c r="E62" s="15"/>
       <c r="F62" s="15"/>
-      <c r="G62" s="191"/>
+      <c r="G62" s="15"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="13" t="s">
@@ -12167,7 +12105,7 @@
       <c r="D63" s="15"/>
       <c r="E63" s="15"/>
       <c r="F63" s="15"/>
-      <c r="G63" s="191" t="s">
+      <c r="G63" s="15" t="s">
         <v>641</v>
       </c>
     </row>
@@ -12180,7 +12118,7 @@
       <c r="D64" s="15"/>
       <c r="E64" s="15"/>
       <c r="F64" s="15"/>
-      <c r="G64" s="191" t="s">
+      <c r="G64" s="15" t="s">
         <v>642</v>
       </c>
     </row>
@@ -12193,7 +12131,7 @@
       <c r="D65" s="15"/>
       <c r="E65" s="15"/>
       <c r="F65" s="15"/>
-      <c r="G65" s="191" t="s">
+      <c r="G65" s="15" t="s">
         <v>413</v>
       </c>
     </row>
@@ -12206,7 +12144,7 @@
       <c r="D66" s="15"/>
       <c r="E66" s="15"/>
       <c r="F66" s="15"/>
-      <c r="G66" s="191"/>
+      <c r="G66" s="15"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -12793,74 +12731,74 @@
       <c r="D1" s="40" t="s">
         <v>265</v>
       </c>
-      <c r="E1" s="173" t="s">
+      <c r="E1" s="172" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="173"/>
-      <c r="G1" s="173"/>
+      <c r="F1" s="172"/>
+      <c r="G1" s="172"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="17"/>
       <c r="B2" s="17"/>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
+      <c r="G2" s="173"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
-      <c r="E3" s="174"/>
-      <c r="F3" s="174"/>
-      <c r="G3" s="174"/>
+      <c r="E3" s="173"/>
+      <c r="F3" s="173"/>
+      <c r="G3" s="173"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="17"/>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
       <c r="D4" s="17"/>
-      <c r="E4" s="174"/>
-      <c r="F4" s="174"/>
-      <c r="G4" s="174"/>
+      <c r="E4" s="173"/>
+      <c r="F4" s="173"/>
+      <c r="G4" s="173"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
-      <c r="E5" s="174"/>
-      <c r="F5" s="174"/>
-      <c r="G5" s="174"/>
+      <c r="E5" s="173"/>
+      <c r="F5" s="173"/>
+      <c r="G5" s="173"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="17"/>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
-      <c r="E6" s="174"/>
-      <c r="F6" s="174"/>
-      <c r="G6" s="174"/>
+      <c r="E6" s="173"/>
+      <c r="F6" s="173"/>
+      <c r="G6" s="173"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
       <c r="D7" s="17"/>
-      <c r="E7" s="174"/>
-      <c r="F7" s="174"/>
-      <c r="G7" s="174"/>
+      <c r="E7" s="173"/>
+      <c r="F7" s="173"/>
+      <c r="G7" s="173"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
-      <c r="E8" s="174"/>
-      <c r="F8" s="174"/>
-      <c r="G8" s="174"/>
+      <c r="E8" s="173"/>
+      <c r="F8" s="173"/>
+      <c r="G8" s="173"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="40" t="s">
@@ -12875,47 +12813,47 @@
       <c r="D10" s="40" t="s">
         <v>269</v>
       </c>
-      <c r="E10" s="173" t="s">
+      <c r="E10" s="172" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="173"/>
-      <c r="G10" s="173"/>
+      <c r="F10" s="172"/>
+      <c r="G10" s="172"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="172"/>
-      <c r="F11" s="172"/>
-      <c r="G11" s="172"/>
+      <c r="E11" s="171"/>
+      <c r="F11" s="171"/>
+      <c r="G11" s="171"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="172"/>
-      <c r="F12" s="172"/>
-      <c r="G12" s="172"/>
+      <c r="E12" s="171"/>
+      <c r="F12" s="171"/>
+      <c r="G12" s="171"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="17"/>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="172"/>
-      <c r="F13" s="172"/>
-      <c r="G13" s="172"/>
+      <c r="E13" s="171"/>
+      <c r="F13" s="171"/>
+      <c r="G13" s="171"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="17"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
-      <c r="E14" s="172"/>
-      <c r="F14" s="172"/>
-      <c r="G14" s="172"/>
+      <c r="E14" s="171"/>
+      <c r="F14" s="171"/>
+      <c r="G14" s="171"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="41" t="s">
@@ -12923,10 +12861,10 @@
       </c>
       <c r="B16" s="39"/>
       <c r="C16" s="12"/>
-      <c r="F16" s="173" t="s">
+      <c r="F16" s="172" t="s">
         <v>271</v>
       </c>
-      <c r="G16" s="173"/>
+      <c r="G16" s="172"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="41" t="s">
@@ -13608,6 +13546,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="22764f65-1f91-4a58-a50d-6cbce21eca12">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2ed2b115-6c2d-4b9d-a375-5d76b684fbe0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009D3D2C266739E043BB3C66B24F8BE822" ma:contentTypeVersion="18" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="9bef219f8659a403fd2b4538d829c5c0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="22764f65-1f91-4a58-a50d-6cbce21eca12" xmlns:ns3="2ed2b115-6c2d-4b9d-a375-5d76b684fbe0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54c6c6508fa9e165dbd1580384fc0569" ns2:_="" ns3:_="">
     <xsd:import namespace="22764f65-1f91-4a58-a50d-6cbce21eca12"/>
@@ -13862,27 +13820,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DCFF404-3738-433F-AD84-3B77DF781E8C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="22764f65-1f91-4a58-a50d-6cbce21eca12"/>
+    <ds:schemaRef ds:uri="2ed2b115-6c2d-4b9d-a375-5d76b684fbe0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="22764f65-1f91-4a58-a50d-6cbce21eca12">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2ed2b115-6c2d-4b9d-a375-5d76b684fbe0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D662CF7-B982-420B-98E9-B390F79A689D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB0A7BAC-FB1D-4FAC-81C3-3C6C450E4559}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13899,23 +13856,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D662CF7-B982-420B-98E9-B390F79A689D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DCFF404-3738-433F-AD84-3B77DF781E8C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="22764f65-1f91-4a58-a50d-6cbce21eca12"/>
-    <ds:schemaRef ds:uri="2ed2b115-6c2d-4b9d-a375-5d76b684fbe0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>